<commit_message>
refactor: tách database vào main để chuẩn bị phân chia app
</commit_message>
<xml_diff>
--- a/URD_v1.xlsx
+++ b/URD_v1.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="72">
   <si>
     <t xml:space="preserve">Danh mục</t>
   </si>
@@ -85,7 +85,7 @@
     <t xml:space="preserve">/api/assets/</t>
   </si>
   <si>
-    <t xml:space="preserve">2. Truy vấn/Xem chi tiết Tài sản</t>
+    <t xml:space="preserve">2. Liệt kê/Xem chi tiết Tài sản</t>
   </si>
   <si>
     <t xml:space="preserve">GET</t>
@@ -109,13 +109,19 @@
     <t xml:space="preserve">/api/assets/&lt;asset_code&gt;/components/</t>
   </si>
   <si>
-    <t xml:space="preserve">5. Quản lý Thanh lý/Hủy</t>
+    <t xml:space="preserve">5. Quản lý Thanh lý/Thu hồi</t>
   </si>
   <si>
     <t xml:space="preserve">PATCH</t>
   </si>
   <si>
     <t xml:space="preserve">/api/assets/&lt;asset_code&gt;/retire/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. Xóa hoàn toàn tài sản</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DELETE</t>
   </si>
   <si>
     <t xml:space="preserve">6. Lấy lịch sử Biến động</t>
@@ -244,6 +250,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -265,11 +272,13 @@
       <sz val="13"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="5">
@@ -339,36 +348,40 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -555,350 +568,365 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="35.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="49.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="23.93"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="33.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="35.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="49.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="23.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="33.24"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4"/>
-      <c r="B3" s="5" t="s">
+      <c r="A3" s="5"/>
+      <c r="B3" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="6" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4"/>
-      <c r="B4" s="5" t="s">
+      <c r="A4" s="5"/>
+      <c r="B4" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="8" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6"/>
-      <c r="B6" s="7" t="s">
+      <c r="A6" s="7"/>
+      <c r="B6" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="8" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6"/>
-      <c r="B7" s="7" t="s">
+      <c r="A7" s="7"/>
+      <c r="B7" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="8" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6"/>
-      <c r="B8" s="7" t="s">
+      <c r="A8" s="7"/>
+      <c r="B8" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="8" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6"/>
-      <c r="B9" s="7" t="s">
+      <c r="A9" s="7"/>
+      <c r="B9" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="8" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6"/>
-      <c r="B10" s="7" t="s">
+      <c r="A10" s="7"/>
+      <c r="B10" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="E10" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7"/>
+      <c r="B11" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="E10" s="7" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="23.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="B11" s="5" t="s">
+      <c r="E11" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="C11" s="5" t="s">
+    </row>
+    <row r="12" customFormat="false" ht="23.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="B12" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D12" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4"/>
-      <c r="B12" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="C12" s="5" t="s">
+      <c r="E12" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="D12" s="5" t="s">
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5"/>
+      <c r="B13" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="D13" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="5" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="23.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4"/>
-      <c r="B13" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="C13" s="5" t="s">
+      <c r="E13" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="D13" s="5" t="s">
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5"/>
+      <c r="B14" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D14" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E13" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4"/>
-      <c r="B14" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="C14" s="5" t="s">
+      <c r="E14" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="D14" s="5" t="s">
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5"/>
+      <c r="B15" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E14" s="5" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="B15" s="7" t="s">
+      <c r="E15" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="C15" s="7" t="s">
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="B16" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="C16" s="8" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6"/>
-      <c r="B16" s="7" t="s">
+      <c r="D16" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="C16" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="D16" s="7" t="s">
+      <c r="E16" s="8" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="7"/>
+      <c r="B17" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="D17" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="E16" s="7" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6"/>
-      <c r="B17" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="C17" s="7" t="s">
+      <c r="E17" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="D17" s="7" t="s">
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="7"/>
+      <c r="B18" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D18" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="E17" s="7" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6"/>
-      <c r="B18" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="C18" s="7" t="s">
+      <c r="E18" s="8" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="7"/>
+      <c r="B19" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="C19" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D19" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="E18" s="7" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="B19" s="5" t="s">
+      <c r="E19" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="C19" s="5" t="s">
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="B20" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="D20" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="E19" s="5" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4"/>
-      <c r="B20" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="C20" s="5" t="s">
+      <c r="E20" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="D20" s="5" t="s">
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5"/>
+      <c r="B21" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="D21" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="E20" s="5" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4"/>
-      <c r="B21" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="C21" s="5" t="s">
+      <c r="E21" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="D21" s="5" t="s">
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5"/>
+      <c r="B22" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="D22" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="E21" s="5" t="s">
-        <v>69</v>
+      <c r="E22" s="6" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A2:A4"/>
-    <mergeCell ref="A5:A10"/>
-    <mergeCell ref="A11:A14"/>
-    <mergeCell ref="A15:A18"/>
-    <mergeCell ref="A19:A21"/>
+    <mergeCell ref="A5:A11"/>
+    <mergeCell ref="A12:A15"/>
+    <mergeCell ref="A16:A19"/>
+    <mergeCell ref="A20:A22"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>